<commit_message>
Product Maintenance and User Access Maintenance documents regenerated: coverage 100% of items and acceptance criteria, notices added to Annex P, configurable points marked for BDOI to confirm the setting
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
@@ -2128,7 +2128,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>BDOI's 90-day alerts, anniversary alerts and recipients (TSU Officer and TSU Team Lead) are kept. v1.1 adds configurable reminder days and the rule that each alert is raised once per alert day (FRPM.004.01). MBS is proposed as an additional recipient, for the set-up of renewals.</t>
+          <t>BDOI's 90-day alerts, anniversary alerts and recipients (TSU Officer and TSU Team Lead) are kept. v1.1 adds configurable reminder days and the rule that each alert is raised once per alert day (FRPM.004.01). MBS is proposed as an additional recipient, for the set-up of renewals. Available in BIBS: the expiry notice period (90 days), the anniversary notice period (90 days) and whether MBS is also told (default: TSU Officers and TSU Team Leads only, as BDOI's text).</t>
         </is>
       </c>
       <c r="H6" s="12" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>BDOI's weekly report of quotation requests is kept and v1.1 adds on-request individual and collective runs (FRPM.007.01). The package creation status asked by BRPM.018 is covered by the new Package Status Update Report (FRPM.007.02).</t>
+          <t>BDOI's weekly report of quotation requests is kept and v1.1 adds on-request individual and collective runs (FRPM.007.01). The package creation status asked by BRPM.018 is covered by the new Package Status Update Report (FRPM.007.02). Available in BIBS: the weekly Consolidated Placement Update Report runs on the day and at the time set (default Thursday 08:00) for a period of days set (default 7) and a scope set (default quotation requests, as BDOI's text); the on-request run is also available.</t>
         </is>
       </c>
       <c r="H7" s="12" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>BDOI's sequential Marketing approval (TL, TH, then UH) is kept. v1.1 adds that no approver approves a request he or she created (FRPM.011.02). BDOI to confirm that every request passes all three levels, or state the levels by market segment or amount.</t>
+          <t>BDOI's sequential Marketing approval (TL, TH, then UH) is kept. v1.1 adds that no approver approves a request he or she created (FRPM.011.02). BDOI to confirm that every request passes all three levels, or state the levels by market segment or amount. Available in BIBS: the Marketing approval chain is a setting: one approval by the Team Leader, Team Head or Unit Head (default, as the BRD), or Team Leader, then Team Head, then Unit Head (BDOI's text).</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>BDOI's direct creation and update of Product Matrix records with Draft and approval is kept. v1.1 adds package versions (FRPM.024.01): the commercial terms of an active package change through a new version, validated before it takes effect, while descriptive details may be edited directly with approval.</t>
+          <t>BDOI's direct creation and update of Product Matrix records with Draft and approval is kept. v1.1 adds package versions (FRPM.024.01): the commercial terms of an active package change through a new version, validated before it takes effect, while descriptive details may be edited directly with approval. Available in BIBS: direct add and update of Product Matrix records with approval is a setting (default on, as BDOI's text); the request route stays available.</t>
         </is>
       </c>
       <c r="H13" s="12" t="inlineStr">
@@ -2848,7 +2848,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>BDOI's deactivation request with an effective date and one approver is kept (FRPM.003.04 to 07). v1.1 adds that nothing is deleted, that incentive rules are flagged for review and that a deactivation advisory is drafted. BDOI to confirm whether a ManCom sign-off is needed for a deactivation.</t>
+          <t>BDOI's deactivation request with an effective date and one approver is kept (FRPM.003.04 to 07). v1.1 adds that nothing is deleted, that incentive rules are flagged for review and that a deactivation advisory is drafted. BDOI to confirm whether a ManCom sign-off is needed for a deactivation. Available in BIBS: the deactivation route is a setting: Deactivate Package with effective date, reason and approver (default, as BDOI's text) or the retirement package request.</t>
         </is>
       </c>
       <c r="H14" s="12" t="inlineStr">
@@ -3478,7 +3478,7 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>BDOI's ManCom routing (selected approvers in parallel, then the President, with e-mail notice) is kept. v1.1 adds that the submitter cannot approve, the optional upload of the signed sheet, the sign-off reference and the locking of the Quotation Slips (FRPM.014.01). BDOI to give the ManCom approver list and confirm the quorum.</t>
+          <t>BDOI's ManCom routing (selected approvers in parallel, then the President, with e-mail notice) is kept. v1.1 adds that the submitter cannot approve, the optional upload of the signed sheet, the sign-off reference and the locking of the Quotation Slips (FRPM.014.01). BDOI to give the ManCom approver list and confirm the quorum. Available in BIBS: the ManCom routing is a setting: the selected approvers approve in parallel, then the President (default, as BDOI's text), or one sign-off; the President is named in the settings.</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
@@ -3748,7 +3748,7 @@
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>BDOI's Request for Deployment step is kept (FRPM.015.01). The BRD (BRPM.015) asks for automatic forwarding to MBS after ManCom approval; v1.1 adds that a deployment request is never possible without the completed ManCom approval and recommends that the deployment request be created automatically on ManCom approval.</t>
+          <t>BDOI's Request for Deployment step is kept (FRPM.015.01). The BRD (BRPM.015) asks for automatic forwarding to MBS after ManCom approval; v1.1 adds that a deployment request is never possible without the completed ManCom approval and recommends that the deployment request be created automatically on ManCom approval. Available in BIBS: the forwarding to MBS is a setting: automatic on the ManCom approval (default, as BRPM.015) or by the Request for Deployment button (BDOI's text).</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="G27" s="12" t="inlineStr">
         <is>
-          <t>BDOI's file names are kept. v1.1 adds the request and slip numbers printed in the documents (PKR-yyyy-nnnnnn, PQS-yyyy-nnnnnn).</t>
+          <t>BDOI's file names are kept. v1.1 adds the request and slip numbers printed in the documents (PKR-yyyy-nnnnnn, PQS-yyyy-nnnnnn). Available in BIBS: BDOI's file names (QS_, ProposalSlip_, PlacementUpdate_, Audit Logs_ with MMDDYYYY) are a setting, on by default.</t>
         </is>
       </c>
       <c r="H27" s="12" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>BDOI's 90-day alerts, anniversary alerts and recipients (TSU Officer and TSU Team Lead) are kept. v1.1 adds configurable reminder days and the rule that each alert is raised once per alert day (FRPM.004.01). MBS is proposed as an additional recipient, for the set-up of renewals.</t>
+          <t>BDOI's 90-day alerts, anniversary alerts and recipients (TSU Officer and TSU Team Lead) are kept. v1.1 adds configurable reminder days and the rule that each alert is raised once per alert day (FRPM.004.01). MBS is proposed as an additional recipient, for the set-up of renewals. Available in BIBS: the expiry notice period (90 days), the anniversary notice period (90 days) and whether MBS is also told (default: TSU Officers and TSU Team Leads only, as BDOI's text).</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -6385,7 +6385,7 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>BDOI's weekly report of quotation requests is kept and v1.1 adds on-request individual and collective runs (FRPM.007.01). The package creation status asked by BRPM.018 is covered by the new Package Status Update Report (FRPM.007.02).</t>
+          <t>BDOI's weekly report of quotation requests is kept and v1.1 adds on-request individual and collective runs (FRPM.007.01). The package creation status asked by BRPM.018 is covered by the new Package Status Update Report (FRPM.007.02). Available in BIBS: the weekly Consolidated Placement Update Report runs on the day and at the time set (default Thursday 08:00) for a period of days set (default 7) and a scope set (default quotation requests, as BDOI's text); the on-request run is also available.</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
@@ -6467,7 +6467,7 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>BDOI's sequential Marketing approval (TL, TH, then UH) is kept. v1.1 adds that no approver approves a request he or she created (FRPM.011.02). BDOI to confirm that every request passes all three levels, or state the levels by market segment or amount.</t>
+          <t>BDOI's sequential Marketing approval (TL, TH, then UH) is kept. v1.1 adds that no approver approves a request he or she created (FRPM.011.02). BDOI to confirm that every request passes all three levels, or state the levels by market segment or amount. Available in BIBS: the Marketing approval chain is a setting: one approval by the Team Leader, Team Head or Unit Head (default, as the BRD), or Team Leader, then Team Head, then Unit Head (BDOI's text).</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
@@ -6631,7 +6631,7 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>BDOI's direct creation and update of Product Matrix records with Draft and approval is kept. v1.1 adds package versions (FRPM.024.01): the commercial terms of an active package change through a new version, validated before it takes effect, while descriptive details may be edited directly with approval.</t>
+          <t>BDOI's direct creation and update of Product Matrix records with Draft and approval is kept. v1.1 adds package versions (FRPM.024.01): the commercial terms of an active package change through a new version, validated before it takes effect, while descriptive details may be edited directly with approval. Available in BIBS: direct add and update of Product Matrix records with approval is a setting (default on, as BDOI's text); the request route stays available.</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
@@ -6672,7 +6672,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>BDOI's deactivation request with an effective date and one approver is kept (FRPM.003.04 to 07). v1.1 adds that nothing is deleted, that incentive rules are flagged for review and that a deactivation advisory is drafted. BDOI to confirm whether a ManCom sign-off is needed for a deactivation.</t>
+          <t>BDOI's deactivation request with an effective date and one approver is kept (FRPM.003.04 to 07). v1.1 adds that nothing is deleted, that incentive rules are flagged for review and that a deactivation advisory is drafted. BDOI to confirm whether a ManCom sign-off is needed for a deactivation. Available in BIBS: the deactivation route is a setting: Deactivate Package with effective date, reason and approver (default, as BDOI's text) or the retirement package request.</t>
         </is>
       </c>
       <c r="F14" s="12" t="inlineStr">
@@ -6959,7 +6959,7 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>BDOI's ManCom routing (selected approvers in parallel, then the President, with e-mail notice) is kept. v1.1 adds that the submitter cannot approve, the optional upload of the signed sheet, the sign-off reference and the locking of the Quotation Slips (FRPM.014.01). BDOI to give the ManCom approver list and confirm the quorum.</t>
+          <t>BDOI's ManCom routing (selected approvers in parallel, then the President, with e-mail notice) is kept. v1.1 adds that the submitter cannot approve, the optional upload of the signed sheet, the sign-off reference and the locking of the Quotation Slips (FRPM.014.01). BDOI to give the ManCom approver list and confirm the quorum. Available in BIBS: the ManCom routing is a setting: the selected approvers approve in parallel, then the President (default, as BDOI's text), or one sign-off; the President is named in the settings.</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -7082,7 +7082,7 @@
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>BDOI's Request for Deployment step is kept (FRPM.015.01). The BRD (BRPM.015) asks for automatic forwarding to MBS after ManCom approval; v1.1 adds that a deployment request is never possible without the completed ManCom approval and recommends that the deployment request be created automatically on ManCom approval.</t>
+          <t>BDOI's Request for Deployment step is kept (FRPM.015.01). The BRD (BRPM.015) asks for automatic forwarding to MBS after ManCom approval; v1.1 adds that a deployment request is never possible without the completed ManCom approval and recommends that the deployment request be created automatically on ManCom approval. Available in BIBS: the forwarding to MBS is a setting: automatic on the ManCom approval (default, as BRPM.015) or by the Request for Deployment button (BDOI's text).</t>
         </is>
       </c>
       <c r="F24" s="12" t="inlineStr">
@@ -7205,7 +7205,7 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>BDOI's file names are kept. v1.1 adds the request and slip numbers printed in the documents (PKR-yyyy-nnnnnn, PQS-yyyy-nnnnnn).</t>
+          <t>BDOI's file names are kept. v1.1 adds the request and slip numbers printed in the documents (PKR-yyyy-nnnnnn, PQS-yyyy-nnnnnn). Available in BIBS: BDOI's file names (QS_, ProposalSlip_, PlacementUpdate_, Audit Logs_ with MMDDYYYY) are a setting, on by default.</t>
         </is>
       </c>
       <c r="F27" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Product Maintenance FRS v1.2 aligned with BIBS: Dashboard, Deactivation Requests, Product Master Transfers, Placement Update Reports, Audit Logs, proposal request and Routing and Approvals screens, updated request list, request form, product and incentive screens, screenshots taken again, settings for the points BDOI decides, schedules, integrations and test cases
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
@@ -2901,7 +2901,7 @@
       </c>
       <c r="T14" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-045.1-01, TC-PM-045.1-02, TC-PM-045.1-03, TC-PM-045.2-01, TC-PM-045.3-01</t>
+          <t>TC-PM-045.4-01, TC-PM-045.4-02, TC-PM-045.1-01, TC-PM-045.1-02, TC-PM-045.1-03</t>
         </is>
       </c>
     </row>
@@ -3531,7 +3531,7 @@
       </c>
       <c r="T21" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01, TC-PM-041.3-01, TC-PM-041.4-01</t>
+          <t>TC-PM-041.5-01, TC-PM-041.5-02, TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="T22" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-033.1-01, TC-PM-033.2-01, TC-PM-033.2-02, TC-PM-033.2-03, TC-PM-033.3-01</t>
+          <t>TC-PM-033.4-01, TC-PM-033.4-02, TC-PM-033.4-03, TC-PM-033.1-01, TC-PM-033.2-01</t>
         </is>
       </c>
     </row>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="T24" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01, TC-PM-041.3-01, TC-PM-041.4-01</t>
+          <t>TC-PM-041.5-01, TC-PM-041.5-02, TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="T36" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-072.1-01, TC-PM-072.1-02, TC-PM-072.2-01, TC-PM-072.1-03, TC-FRPM.029.01-AC1</t>
+          <t>TC-PM-072.1-01, TC-PM-072.1-02, TC-PM-072.2-01, TC-PM-072.2-02, TC-PM-072.1-03</t>
         </is>
       </c>
     </row>
@@ -5421,7 +5421,7 @@
       </c>
       <c r="T42" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01, TC-PM-041.3-01, TC-PM-041.4-01</t>
+          <t>TC-PM-041.5-01, TC-PM-041.5-02, TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01</t>
         </is>
       </c>
     </row>
@@ -5691,7 +5691,7 @@
       </c>
       <c r="T45" s="12" t="inlineStr">
         <is>
-          <t>TC-PM-005.1-01, TC-PM-005.2-01, TC-PM-005.3-01, TC-FRPM.021.01-AC1, TC-FRPM.021.01-AC2</t>
+          <t>TC-PM-005.4-01, TC-PM-005.1-01, TC-PM-005.2-01, TC-PM-005.3-01, TC-PM-SCR-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Product Maintenance FRS v1.3: simplified and end-to-end swimlane process flows (flows/brd03, reproducible), points beyond the BRD coloured (8 green available in BIBS, 5 orange change requests), section 1.5 How to Read, Annex Y with change requests and effort, green points and the BRD line check, Annex T rows T-18 to T-21 (BRD maintenance and disaster lines, programme NFRs 10.07 and 4.03); CR effort workbook (30 man-days), CR register and RTM linked; review copy shades the changes of v1.3
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
+++ b/docs/deliverables/out/Programme/BDOI_Template_FRS/BRD-03_Product_Maintenance/BIBS_CR_BRD-03_Change_Request_Register_v1.0.xlsx
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'README'!$A$4:$D$35</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'README'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Register'!$A$4:$T$53</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Register'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Decisions log'!$A$4:$K$82</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Decisions log'!$4:$4</definedName>
@@ -753,7 +753,7 @@
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>BRD-03 Product Maintenance – changes after the sign-off of the FRS v1.2</t>
+          <t>BRD-03 Product Maintenance – changes after the sign-off of the FRS v1.3</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>Number in Annex M of the FRS v1.2</t>
+          <t>Number in Annex M of the FRS v1.3</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr"/>
@@ -1656,7 +1656,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Signing the FRS v1.2 freezes its requirements (FRS Annex W). A change after sign-off follows the steps below.</t>
+          <t>Signing the FRS v1.3 freezes its requirements (FRS Annex W). A change after sign-off follows the steps below.</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:T53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5965,32 +5965,482 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="12" t="inlineStr">
+        <is>
+          <t>CR-PM-101</t>
+        </is>
+      </c>
+      <c r="B49" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D49" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.012 (extends)</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>FRPM.006.01, FRPM.012.01; Annex P NT-16; FRS Annex Y.2</t>
+        </is>
+      </c>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Quotation Slip decision notice to the preparer</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>The TSU Officer who prepares a Quotation Slip learns of its approval or return only by opening the request; the notice lets the slip go to the insurers the same day.</t>
+        </is>
+      </c>
+      <c r="H49" s="12" t="inlineStr">
+        <is>
+          <t>Proposal beyond the BRD text</t>
+        </is>
+      </c>
+      <c r="I49" s="12" t="inlineStr">
+        <is>
+          <t>Not available: the slip approval (negotiation service) sends the slip to the insurers but no notice to the preparer; the notice service of the platform is available and is reused.</t>
+        </is>
+      </c>
+      <c r="J49" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved by 30-Nov-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="12" t="inlineStr">
+        <is>
+          <t>3.5 (BIBS_CR_BRD-03_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L49" s="12" t="inlineStr">
+        <is>
+          <t>Notice service and e-mail channel (Annex S, IN-08)</t>
+        </is>
+      </c>
+      <c r="M49" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N49" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O49" s="27" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P49" s="12" t="n"/>
+      <c r="Q49" s="12" t="n"/>
+      <c r="R49" s="28" t="n"/>
+      <c r="S49" s="12" t="inlineStr">
+        <is>
+          <t>Drop 1</t>
+        </is>
+      </c>
+      <c r="T49" s="12" t="inlineStr">
+        <is>
+          <t>TC-PM-013.1-01, TC-PM-013.2-01, TC-PM-013.3-01, TC-PM-030.1-01, TC-PM-030.2-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t>CR-PM-102</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D50" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.015 (extends)</t>
+        </is>
+      </c>
+      <c r="E50" s="12" t="inlineStr">
+        <is>
+          <t>FRPM.014.01; Annex P NT-13, NT-14; FRS Annex Y.2</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>ManCom e-mails in BDOI's wording, with the President's text</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's FRS asks for the ManCom approval e-mail in its own wording and a separate text when the request reaches the President.</t>
+        </is>
+      </c>
+      <c r="H50" s="12" t="inlineStr">
+        <is>
+          <t>Proposal beyond the BRD text</t>
+        </is>
+      </c>
+      <c r="I50" s="12" t="inlineStr">
+        <is>
+          <t>Partly available: each ManCom approver is told in the system with an e-mail copy, in one standard text; the two BDOI texts are to be added.</t>
+        </is>
+      </c>
+      <c r="J50" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved by 30-Nov-2026</t>
+        </is>
+      </c>
+      <c r="K50" s="12" t="inlineStr">
+        <is>
+          <t>2.5 (BIBS_CR_BRD-03_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L50" s="12" t="inlineStr">
+        <is>
+          <t>E-mail channel of BDOI (Annex S, IN-08)</t>
+        </is>
+      </c>
+      <c r="M50" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N50" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O50" s="27" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P50" s="12" t="n"/>
+      <c r="Q50" s="12" t="n"/>
+      <c r="R50" s="28" t="n"/>
+      <c r="S50" s="12" t="inlineStr">
+        <is>
+          <t>Drop 1</t>
+        </is>
+      </c>
+      <c r="T50" s="12" t="inlineStr">
+        <is>
+          <t>TC-PM-041.5-01, TC-PM-041.5-02, TC-PM-041.1-01, TC-PM-041.1-02, TC-PM-041.2-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>CR-PM-103</t>
+        </is>
+      </c>
+      <c r="B51" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C51" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D51" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.024 (extends)</t>
+        </is>
+      </c>
+      <c r="E51" s="12" t="inlineStr">
+        <is>
+          <t>FRPM.021.01, FRPM.021.02; Annex M.5; FRS Annex Y.2</t>
+        </is>
+      </c>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Old and new field values of product master changes in the audit log</t>
+        </is>
+      </c>
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.024 asks for the audit trail of every action; the auditors also expect to see, for a changed master record, which field changed from which value to which value.</t>
+        </is>
+      </c>
+      <c r="H51" s="12" t="inlineStr">
+        <is>
+          <t>Proposal beyond the BRD text</t>
+        </is>
+      </c>
+      <c r="I51" s="12" t="inlineStr">
+        <is>
+          <t>Partly available: every create, change and authorize of a product master is in the audit log with user and time; the field-by-field old and new values are kept today for package terms only.</t>
+        </is>
+      </c>
+      <c r="J51" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved by 30-Nov-2026</t>
+        </is>
+      </c>
+      <c r="K51" s="12" t="inlineStr">
+        <is>
+          <t>9 (BIBS_CR_BRD-03_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L51" s="12" t="inlineStr">
+        <is>
+          <t>Audit log of the platform (old and new value columns exist)</t>
+        </is>
+      </c>
+      <c r="M51" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N51" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O51" s="27" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P51" s="12" t="n"/>
+      <c r="Q51" s="12" t="n"/>
+      <c r="R51" s="28" t="n"/>
+      <c r="S51" s="12" t="inlineStr">
+        <is>
+          <t>Drop 1</t>
+        </is>
+      </c>
+      <c r="T51" s="12" t="inlineStr">
+        <is>
+          <t>TC-PM-005.4-01, TC-PM-005.1-01, TC-PM-005.2-01, TC-PM-005.3-01, TC-PM-SCR-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>CR-PM-104</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D52" s="12" t="inlineStr">
+        <is>
+          <t>Not in BRD</t>
+        </is>
+      </c>
+      <c r="E52" s="12" t="inlineStr">
+        <is>
+          <t>Annex T, T-15; FRS Annex Y.2</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Accessibility of the Product Maintenance screens (WCAG 2.2 level AA)</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>No BDOI BRD asks for an accessibility level; the programme register proposes WCAG 2.2 AA so that keyboard and screen-reader users can work in the module.</t>
+        </is>
+      </c>
+      <c r="H52" s="12" t="inlineStr">
+        <is>
+          <t>Proposal beyond the BRD text</t>
+        </is>
+      </c>
+      <c r="I52" s="12" t="inlineStr">
+        <is>
+          <t>Partly available: the screens use the platform components and are usable with the keyboard; no WCAG 2.2 AA conformance check has been made on the module (about 8 of 35 screen files carry accessibility labels).</t>
+        </is>
+      </c>
+      <c r="J52" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved by 30-Nov-2026</t>
+        </is>
+      </c>
+      <c r="K52" s="12" t="inlineStr">
+        <is>
+          <t>11.5 (BIBS_CR_BRD-03_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L52" s="12" t="inlineStr">
+        <is>
+          <t>BDOI's decision on the accessibility level (Annex V, PQ18)</t>
+        </is>
+      </c>
+      <c r="M52" s="12" t="inlineStr">
+        <is>
+          <t>Test cases to add for the change</t>
+        </is>
+      </c>
+      <c r="N52" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="O52" s="27" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P52" s="12" t="n"/>
+      <c r="Q52" s="12" t="n"/>
+      <c r="R52" s="28" t="n"/>
+      <c r="S52" s="12" t="inlineStr">
+        <is>
+          <t>Drop 1</t>
+        </is>
+      </c>
+      <c r="T52" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>CR-PM-105</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>11-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C53" s="12" t="inlineStr">
+        <is>
+          <t>iorta TechNXT Project Team</t>
+        </is>
+      </c>
+      <c r="D53" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.021 (extends)</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>FRPM.001.01; FRS Annex Y.2</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>'Due soon' marker at 80% of the stage service level</t>
+        </is>
+      </c>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>BRPM.021 asks that each approval step is completed within the defined service level; an amber marker relative to each stage's own service level warns before the breach on short and long stages alike.</t>
+        </is>
+      </c>
+      <c r="H53" s="12" t="inlineStr">
+        <is>
+          <t>Proposal beyond the BRD text</t>
+        </is>
+      </c>
+      <c r="I53" s="12" t="inlineStr">
+        <is>
+          <t>Partly available: a request is marked 'due soon' when it is due within 8 hours, whatever the service level of the stage; overdue (red) is available.</t>
+        </is>
+      </c>
+      <c r="J53" s="12" t="inlineStr">
+        <is>
+          <t>Within the drop if approved by 30-Nov-2026</t>
+        </is>
+      </c>
+      <c r="K53" s="12" t="inlineStr">
+        <is>
+          <t>3.5 (BIBS_CR_BRD-03_Effort_Estimate_v1.0.xlsx)</t>
+        </is>
+      </c>
+      <c r="L53" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M53" s="12" t="inlineStr">
+        <is>
+          <t>Update the linked test cases</t>
+        </is>
+      </c>
+      <c r="N53" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O53" s="27" t="inlineStr">
+        <is>
+          <t>Candidate - for decision</t>
+        </is>
+      </c>
+      <c r="P53" s="12" t="n"/>
+      <c r="Q53" s="12" t="n"/>
+      <c r="R53" s="28" t="n"/>
+      <c r="S53" s="12" t="inlineStr">
+        <is>
+          <t>Drop 1</t>
+        </is>
+      </c>
+      <c r="T53" s="12" t="inlineStr">
+        <is>
+          <t>TC-PM-070.1-01, TC-PM-070.1-02, TC-PM-070.2-01, TC-PM-070.3-01, TC-PM-070.3-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:T48"/>
+  <autoFilter ref="A4:T53"/>
   <mergeCells count="1">
     <mergeCell ref="A2:T2"/>
   </mergeCells>
-  <conditionalFormatting sqref="O5:O548">
+  <conditionalFormatting sqref="O5:O553">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0" stopIfTrue="1">
       <formula>"Closed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A5:T548">
+  <conditionalFormatting sqref="A5:T553">
     <cfRule type="expression" priority="2" dxfId="1">
       <formula>AND(MOD(ROW(),2)=0,$A5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation sqref="H5:H548" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
+    <dataValidation sqref="H5:H553" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Type" error="Choose a value from the list (Type)." type="list">
       <formula1>'Lists'!$A$2:$A$9</formula1>
     </dataValidation>
-    <dataValidation sqref="N5:N548" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
+    <dataValidation sqref="N5:N553" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Priority" error="Choose a value from the list (Priority)." type="list">
       <formula1>'Lists'!$B$2:$B$4</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O548" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
+    <dataValidation sqref="O5:O553" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Status" error="Choose a value from the list (Status)." type="list">
       <formula1>'Lists'!$C$2:$C$10</formula1>
     </dataValidation>
-    <dataValidation sqref="S5:S548" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Target drop" error="Choose a value from the list (Target drop)." type="list">
+    <dataValidation sqref="S5:S553" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Target drop" error="Choose a value from the list (Target drop)." type="list">
       <formula1>'Lists'!$D$2:$D$6</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>